<commit_message>
Manente v2 — pós interna, estúdio a 3.000/diária, design com a agência
Lucro cai de 16.274 para 4.274 (6,5%). A pós interna e o design do painel
zeraram seis linhas, mas o custo interno do estúdio — 4 diárias × 3.000 —
comeu mais do que elas devolveram.

Sobram R$ 4.274 para dez linhas ainda sem valor. Cinco pessoas × 4 diárias a
R$ 500 já levam o job a prejuízo. Está dito na skill nesses termos.

Dois números registrados como conhecimento da casa: o Estúdio Morumbi custa
R$ 3.000 a diária internamente, e essa cobrança é transferência entre unidades
— o job mostra 4.274 e o grupo fica com 16.274. Os dois precisam ser ditos
juntos, senão um deles engana.

O AI-Driven Design do painel está na proposta como entrega da YAD e a MDias
assumiu. Ficou na observação da linha: se voltarem a pedir, é mudança de
escopo, não cortesia.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NubHinCg53tN7sLp5QNqJV
</commit_message>
<xml_diff>
--- a/producao/pressupostos/PRESSUPOSTO_REAL_MANENTE_LED.xlsx
+++ b/producao/pressupostos/PRESSUPOSTO_REAL_MANENTE_LED.xlsx
@@ -791,7 +791,7 @@
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>v1</t>
+          <t>v2</t>
         </is>
       </c>
       <c r="D13" s="8" t="n"/>
@@ -2090,20 +2090,18 @@
       <c r="E18" s="15" t="n">
         <v>9</v>
       </c>
-      <c r="F18" s="16" t="n"/>
+      <c r="F18" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="G18" s="36">
         <f>IF(OR(E18="",F18=""),"",ROUND(E18*F18,2))</f>
         <v/>
       </c>
-      <c r="H18" s="15" t="inlineStr">
-        <is>
-          <t>A PAGAR</t>
-        </is>
-      </c>
+      <c r="H18" s="15" t="inlineStr"/>
       <c r="I18" s="14" t="n"/>
       <c r="J18" s="12" t="inlineStr">
         <is>
-          <t>ADICIONADO — teto do escopo: 15 min finalizados ou 72h de ilha, o que vier primeiro</t>
+          <t>pós interna da YAD — sem custo de terceiro. Se alguém receber cachê por este job, lançar aqui.</t>
         </is>
       </c>
     </row>
@@ -2126,20 +2124,18 @@
       <c r="E19" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="16" t="n"/>
+      <c r="F19" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="G19" s="36">
         <f>IF(OR(E19="",F19=""),"",ROUND(E19*F19,2))</f>
         <v/>
       </c>
-      <c r="H19" s="15" t="inlineStr">
-        <is>
-          <t>A PAGAR</t>
-        </is>
-      </c>
+      <c r="H19" s="15" t="inlineStr"/>
       <c r="I19" s="14" t="n"/>
       <c r="J19" s="12" t="inlineStr">
         <is>
-          <t>ADICIONADO — prometido no escopo</t>
+          <t>pós interna da YAD — sem custo de terceiro. Se alguém receber cachê por este job, lançar aqui.</t>
         </is>
       </c>
     </row>
@@ -2162,20 +2158,18 @@
       <c r="E20" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="16" t="n"/>
+      <c r="F20" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="G20" s="36">
         <f>IF(OR(E20="",F20=""),"",ROUND(E20*F20,2))</f>
         <v/>
       </c>
-      <c r="H20" s="15" t="inlineStr">
-        <is>
-          <t>A PAGAR</t>
-        </is>
-      </c>
+      <c r="H20" s="15" t="inlineStr"/>
       <c r="I20" s="14" t="n"/>
       <c r="J20" s="12" t="inlineStr">
         <is>
-          <t>ADICIONADO — prometido no escopo</t>
+          <t>pós interna da YAD — sem custo de terceiro. Se alguém receber cachê por este job, lançar aqui.</t>
         </is>
       </c>
     </row>
@@ -2198,20 +2192,18 @@
       <c r="E21" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="16" t="n"/>
+      <c r="F21" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="G21" s="36">
         <f>IF(OR(E21="",F21=""),"",ROUND(E21*F21,2))</f>
         <v/>
       </c>
-      <c r="H21" s="15" t="inlineStr">
-        <is>
-          <t>A PAGAR</t>
-        </is>
-      </c>
+      <c r="H21" s="15" t="inlineStr"/>
       <c r="I21" s="14" t="n"/>
       <c r="J21" s="12" t="inlineStr">
         <is>
-          <t>ADICIONADO — prometido no escopo</t>
+          <t>pós interna da YAD — sem custo de terceiro. Se alguém receber cachê por este job, lançar aqui.</t>
         </is>
       </c>
     </row>
@@ -2234,20 +2226,18 @@
       <c r="E22" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="16" t="n"/>
+      <c r="F22" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="G22" s="36">
         <f>IF(OR(E22="",F22=""),"",ROUND(E22*F22,2))</f>
         <v/>
       </c>
-      <c r="H22" s="15" t="inlineStr">
-        <is>
-          <t>A PAGAR</t>
-        </is>
-      </c>
+      <c r="H22" s="15" t="inlineStr"/>
       <c r="I22" s="14" t="n"/>
       <c r="J22" s="12" t="inlineStr">
         <is>
-          <t>ADICIONADO — prometido no escopo</t>
+          <t>pós interna da YAD — sem custo de terceiro. Se alguém receber cachê por este job, lançar aqui.</t>
         </is>
       </c>
     </row>
@@ -2270,20 +2260,18 @@
       <c r="E23" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="16" t="n"/>
+      <c r="F23" s="13" t="n">
+        <v>0</v>
+      </c>
       <c r="G23" s="36">
         <f>IF(OR(E23="",F23=""),"",ROUND(E23*F23,2))</f>
         <v/>
       </c>
-      <c r="H23" s="15" t="inlineStr">
-        <is>
-          <t>A PAGAR</t>
-        </is>
-      </c>
+      <c r="H23" s="15" t="inlineStr"/>
       <c r="I23" s="14" t="n"/>
       <c r="J23" s="12" t="inlineStr">
         <is>
-          <t>ADICIONADO — criação visual do LED dentro da linguagem aprovada; 3D e produção virtual ficam fora</t>
+          <t>a MDias faz o design do painel — sem custo para a YAD. ATENÇÃO: a proposta lista isso como escopo da YAD; se voltarem a pedir, é mudança de escopo.</t>
         </is>
       </c>
     </row>
@@ -2307,17 +2295,21 @@
         <v>4</v>
       </c>
       <c r="F24" s="13" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="G24" s="36">
         <f>IF(OR(E24="",F24=""),"",ROUND(E24*F24,2))</f>
         <v/>
       </c>
-      <c r="H24" s="15" t="inlineStr"/>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>A PAGAR</t>
+        </is>
+      </c>
       <c r="I24" s="14" t="n"/>
       <c r="J24" s="12" t="inlineStr">
         <is>
-          <t>unidade própria da YAD — decidir se entra custo interno de ocupação</t>
+          <t>custo interno de ocupação, R$ 3.000 por diária — transferência entre YAD produção e a unidade</t>
         </is>
       </c>
     </row>

</xml_diff>